<commit_message>
update: menambahkan pilihan status ekonomi di tambah data warga
</commit_message>
<xml_diff>
--- a/public/template_import_warga.xlsx
+++ b/public/template_import_warga.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,8 +54,18 @@
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <i val="1"/>
+      <color rgb="00888888"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -92,6 +102,11 @@
         <fgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001a6b3c"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -119,7 +134,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -151,6 +166,15 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -696,6 +720,7 @@
     <col width="22" customWidth="1" min="14" max="14"/>
     <col width="18" customWidth="1" min="15" max="15"/>
     <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="18" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
@@ -709,7 +734,13 @@
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>⚠️  PETUNJUK PENGISIAN:
-• NIK wajib 16 digit angka  • NO_KK harus sudah terdaftar (upload Data KK lebih dulu)  • TANGGAL_LAHIR format: YYYY-MM-DD (contoh: 1990-05-25)  • STATUS_TINGGAL: domisili_asli / non_ktp / sementara / non_domisili  • JENIS_KELAMIN: Laki-laki / Perempuan  • Hapus baris contoh sebelum upload</t>
+• NIK wajib 16 digit angka
+• NO_KK harus sudah terdaftar (upload Data KK lebih dulu)
+• TANGGAL_LAHIR format: YYYY-MM-DD (contoh: 1990-05-25)
+• JENIS_KELAMIN: Laki-laki / Perempuan
+• STATUS_TINGGAL: domisili_asli / non_ktp / sementara / non_domisili
+• STATUS_EKONOMI: mampu / rentan_miskin / tidak_mampu / miskin / sangat_miskin
+• Kolom bertanda * WAJIB diisi  •  Hapus baris contoh (baris 4-5) sebelum upload  •  Format file tetap .xlsx</t>
         </is>
       </c>
     </row>
@@ -794,6 +825,11 @@
           <t>KEWARGANEGARAAN</t>
         </is>
       </c>
+      <c r="Q3" s="13" t="inlineStr">
+        <is>
+          <t>STATUS_EKONOMI</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -874,6 +910,11 @@
       <c r="P4" s="4" t="inlineStr">
         <is>
           <t>WNI</t>
+        </is>
+      </c>
+      <c r="Q4" s="11" t="inlineStr">
+        <is>
+          <t>mampu</t>
         </is>
       </c>
     </row>
@@ -948,6 +989,11 @@
       <c r="P5" s="5" t="inlineStr">
         <is>
           <t>WNI</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>rentan_miskin</t>
         </is>
       </c>
     </row>
@@ -1108,7 +1154,7 @@
     <mergeCell ref="A2:R2"/>
     <mergeCell ref="A1:R1"/>
   </mergeCells>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation sqref="F4:F1003" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Laki-laki,Perempuan"</formula1>
     </dataValidation>
@@ -1133,6 +1179,9 @@
     <dataValidation sqref="P4:P1003" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"WNI,WNA"</formula1>
     </dataValidation>
+    <dataValidation sqref="Q4:Q1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nilai tidak valid" error="Pilih: mampu / rentan_miskin / tidak_mampu / miskin / sangat_miskin" type="list">
+      <formula1>"mampu,rentan_miskin,tidak_mampu,miskin,sangat_miskin"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1144,7 +1193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D59"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1158,6 +1207,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
@@ -1194,6 +1244,7 @@
         </is>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
@@ -1278,6 +1329,7 @@
         </is>
       </c>
     </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
@@ -1386,6 +1438,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="9" t="inlineStr">
         <is>
@@ -1446,6 +1499,7 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
@@ -1554,6 +1608,7 @@
         </is>
       </c>
     </row>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
@@ -1662,6 +1717,7 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
@@ -1722,6 +1778,7 @@
         </is>
       </c>
     </row>
+    <row r="56"/>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
@@ -1758,6 +1815,83 @@
         </is>
       </c>
     </row>
+    <row r="60"/>
+    <row r="61">
+      <c r="A61" s="14" t="inlineStr">
+        <is>
+          <t>STATUS_EKONOMI</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>Nilai Yang Diizinkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>STATUS_EKONOMI</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>mampu</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>STATUS_EKONOMI</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>rentan_miskin</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>STATUS_EKONOMI</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>tidak_mampu</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>STATUS_EKONOMI</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>miskin</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>STATUS_EKONOMI</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>sangat_miskin</t>
+        </is>
+      </c>
+    </row>
+    <row r="68"/>
+    <row r="69"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
update: menaghilangkan status sangat miskin dan rentan miskin di status ekonomi
</commit_message>
<xml_diff>
--- a/public/template_import_warga.xlsx
+++ b/public/template_import_warga.xlsx
@@ -739,7 +739,7 @@
 • TANGGAL_LAHIR format: YYYY-MM-DD (contoh: 1990-05-25)
 • JENIS_KELAMIN: Laki-laki / Perempuan
 • STATUS_TINGGAL: domisili_asli / non_ktp / sementara / non_domisili
-• STATUS_EKONOMI: mampu / rentan_miskin / tidak_mampu / miskin / sangat_miskin
+• STATUS_EKONOMI: mampu / rentan_miskin / miskin
 • Kolom bertanda * WAJIB diisi  •  Hapus baris contoh (baris 4-5) sebelum upload  •  Format file tetap .xlsx</t>
         </is>
       </c>
@@ -1193,7 +1193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D69"/>
+  <dimension ref="A1:D72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1862,36 +1862,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>tidak_mampu</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>STATUS_EKONOMI</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
           <t>miskin</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>STATUS_EKONOMI</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>sangat_miskin</t>
-        </is>
-      </c>
-    </row>
+    <row r="66"/>
+    <row r="67"/>
     <row r="68"/>
     <row r="69"/>
+    <row r="70"/>
+    <row r="71"/>
+    <row r="72"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>

</xml_diff>

<commit_message>
update: update dashboard dan input status hubungan baru
</commit_message>
<xml_diff>
--- a/public/template_import_warga.xlsx
+++ b/public/template_import_warga.xlsx
@@ -1,54 +1,31 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Petunjuk" sheetId="1" r:id="rId1"/>
-    <sheet name="Data KK" sheetId="2" r:id="rId2"/>
-    <sheet name="Data Warga" sheetId="3" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Petunjuk" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data KK" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Warga" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
+  <definedNames/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
-</file>
-
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
-      <sz val="12"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="12"/>
       <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill patternType="none"/>
+      <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -67,13 +44,80 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -398,331 +442,474 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="80.83203125" customWidth="1"/>
+    <col width="80.83203125" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>TEMPLATE IMPORT DATA WARGA</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TEMPLATE IMPORT DATA WARGA</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>Sistem Administrasi Dukuh Majegan, Pandowoharjo, Sleman</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sistem Administrasi Dukuh Majegan, Pandowoharjo, Sleman</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>PETUNJUK PENGISIAN:</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>PETUNJUK PENGISIAN:</t>
+        </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
-        <v>1. Isi data di sheet "Data Warga" mulai baris ke-4 (baris 1-3 adalah header)</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1. Isi data di sheet "Data Warga" mulai baris ke-4 (baris 1-3 adalah header)</t>
+        </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="str">
-        <v>2. Kolom bertanda * WAJIB diisi</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2. Kolom bertanda * WAJIB diisi</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="str">
-        <v>3. NIK harus 16 digit angka</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>3. NIK harus 16 digit angka</t>
+        </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="str">
-        <v>4. NO_KK harus sudah terdaftar di sheet "Data KK" atau di database</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>4. NO_KK harus sudah terdaftar di sheet "Data KK" atau di database</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="str">
-        <v>5. JENIS_KELAMIN: Laki-laki / Perempuan</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>5. JENIS_KELAMIN: Laki-laki / Perempuan</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="str">
-        <v>6. STATUS_TINGGAL: domisili_asli / non_ktp / sementara / non_domisili</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>6. STATUS_TINGGAL: domisili_asli / non_ktp / sementara / non_domisili</t>
+        </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="str">
-        <v>7. STATUS_EKONOMI: mampu / rentan_miskin / miskin</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>7. STATUS_EKONOMI: mampu / rentan_miskin / miskin</t>
+        </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="str">
-        <v>8. GOLONGAN_DARAH: A / B / AB / O (kosongkan jika tidak tahu)</v>
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>8. GOLONGAN_DARAH: A / B / AB / O (kosongkan jika tidak tahu)</t>
+        </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="str">
-        <v>9. AGAMA: Islam / Kristen / Katolik / Hindu / Buddha / Konghucu</v>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>9. AGAMA: Islam / Kristen / Katolik / Hindu / Buddha / Konghucu</t>
+        </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="str">
-        <v>10. TANGGAL_LAHIR format: YYYY-MM-DD (contoh: 1990-05-17)</v>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>10. TANGGAL_LAHIR format: YYYY-MM-DD (contoh: 1990-05-17)</t>
+        </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="str">
-        <v>11. STATUS_HUBUNGAN: Kepala Keluarga / Istri / Anak / Famili Lain / Pembantu</v>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>11. STATUS_HUBUNGAN: Kepala Keluarga / Istri / Anak / Orang Tua / Famili Lain / Pembantu</t>
+        </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="str">
-        <v>12. ALAMAT_KTP: Alamat lengkap sesuai tertera di KTP (opsional)</v>
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>12. ALAMAT_KTP: Alamat lengkap sesuai tertera di KTP (opsional)</t>
+        </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="str">
-        <v>13. ALAMAT_DOMISILI: Isi bila alamat domisili berbeda dengan KTP (opsional)</v>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>13. ALAMAT_DOMISILI: Isi bila alamat domisili berbeda dengan KTP (opsional)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A17"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:G4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="40.83203125" customWidth="1"/>
-    <col min="4" max="4" width="5.83203125" customWidth="1"/>
-    <col min="5" max="5" width="5.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-    <col min="7" max="7" width="15.83203125" customWidth="1"/>
+    <col width="20.83203125" customWidth="1" min="1" max="1"/>
+    <col width="30.83203125" customWidth="1" min="2" max="2"/>
+    <col width="40.83203125" customWidth="1" min="3" max="3"/>
+    <col width="5.83203125" customWidth="1" min="4" max="4"/>
+    <col width="5.83203125" customWidth="1" min="5" max="5"/>
+    <col width="12.83203125" customWidth="1" min="6" max="6"/>
+    <col width="15.83203125" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>TEMPLATE DATA KARTU KELUARGA — isi KK terlebih dahulu sebelum import warga</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TEMPLATE DATA KARTU KELUARGA — isi KK terlebih dahulu sebelum import warga</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>Sistem Administrasi Dukuh Majegan</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sistem Administrasi Dukuh Majegan</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>NO_KK *</v>
-      </c>
-      <c r="B3" t="str">
-        <v>NAMA_KEPALA *</v>
-      </c>
-      <c r="C3" t="str">
-        <v>ALAMAT *</v>
-      </c>
-      <c r="D3" t="str">
-        <v>RT</v>
-      </c>
-      <c r="E3" t="str">
-        <v>RW</v>
-      </c>
-      <c r="F3" t="str">
-        <v>DUSUN</v>
-      </c>
-      <c r="G3" t="str">
-        <v>TELEPON</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NO_KK *</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NAMA_KEPALA *</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>ALAMAT *</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>DUSUN</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>TELEPON</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>3404051234567890</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Ahmad Suharto</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Dusun Majegan RT 01 RW 01</v>
-      </c>
-      <c r="D4" t="str">
-        <v>01</v>
-      </c>
-      <c r="E4" t="str">
-        <v>01</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Majegan</v>
-      </c>
-      <c r="G4" t="str">
-        <v>08123456789</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3404051234567890</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ahmad Suharto</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Dusun Majegan RT 01 RW 01</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Majegan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>08123456789</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:S4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="20.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="14.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-    <col min="7" max="7" width="10.83203125" customWidth="1"/>
-    <col min="8" max="8" width="15.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
-    <col min="11" max="11" width="18.83203125" customWidth="1"/>
-    <col min="12" max="12" width="10.83203125" customWidth="1"/>
-    <col min="13" max="13" width="15.83203125" customWidth="1"/>
-    <col min="14" max="14" width="25.83203125" customWidth="1"/>
-    <col min="15" max="15" width="12.83203125" customWidth="1"/>
-    <col min="16" max="16" width="16.83203125" customWidth="1"/>
-    <col min="17" max="17" width="14.83203125" customWidth="1"/>
-    <col min="18" max="18" width="45.83203125" customWidth="1"/>
-    <col min="19" max="19" width="45.83203125" customWidth="1"/>
+    <col width="20.83203125" customWidth="1" min="1" max="1"/>
+    <col width="20.83203125" customWidth="1" min="2" max="2"/>
+    <col width="30.83203125" customWidth="1" min="3" max="3"/>
+    <col width="15.83203125" customWidth="1" min="4" max="4"/>
+    <col width="14.83203125" customWidth="1" min="5" max="5"/>
+    <col width="14.83203125" customWidth="1" min="6" max="6"/>
+    <col width="10.83203125" customWidth="1" min="7" max="7"/>
+    <col width="15.83203125" customWidth="1" min="8" max="8"/>
+    <col width="18.83203125" customWidth="1" min="9" max="9"/>
+    <col width="16.83203125" customWidth="1" min="10" max="10"/>
+    <col width="18.83203125" customWidth="1" min="11" max="11"/>
+    <col width="10.83203125" customWidth="1" min="12" max="12"/>
+    <col width="15.83203125" customWidth="1" min="13" max="13"/>
+    <col width="25.83203125" customWidth="1" min="14" max="14"/>
+    <col width="12.83203125" customWidth="1" min="15" max="15"/>
+    <col width="16.83203125" customWidth="1" min="16" max="16"/>
+    <col width="14.83203125" customWidth="1" min="17" max="17"/>
+    <col width="45.83203125" customWidth="1" min="18" max="18"/>
+    <col width="45.83203125" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="str">
-        <v>TEMPLATE DATA WARGA — pastikan NO_KK sudah terdaftar di sheet Data KK atau database</v>
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>TEMPLATE DATA WARGA — pastikan NO_KK sudah terdaftar di sheet Data KK atau database</t>
+        </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>Sistem Administrasi Dukuh Majegan</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Sistem Administrasi Dukuh Majegan</t>
+        </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>NIK *</v>
-      </c>
-      <c r="B3" t="str">
-        <v>NO_KK *</v>
-      </c>
-      <c r="C3" t="str">
-        <v>NAMA_LENGKAP *</v>
-      </c>
-      <c r="D3" t="str">
-        <v>TEMPAT_LAHIR</v>
-      </c>
-      <c r="E3" t="str">
-        <v>TANGGAL_LAHIR</v>
-      </c>
-      <c r="F3" t="str">
-        <v>JENIS_KELAMIN *</v>
-      </c>
-      <c r="G3" t="str">
-        <v>AGAMA</v>
-      </c>
-      <c r="H3" t="str">
-        <v>PENDIDIKAN</v>
-      </c>
-      <c r="I3" t="str">
-        <v>PEKERJAAN</v>
-      </c>
-      <c r="J3" t="str">
-        <v>STATUS_PERKAWINAN</v>
-      </c>
-      <c r="K3" t="str">
-        <v>STATUS_HUBUNGAN *</v>
-      </c>
-      <c r="L3" t="str">
-        <v>GOLONGAN_DARAH</v>
-      </c>
-      <c r="M3" t="str">
-        <v>TELEPON</v>
-      </c>
-      <c r="N3" t="str">
-        <v>EMAIL</v>
-      </c>
-      <c r="O3" t="str">
-        <v>KEWARGANEGARAAN</v>
-      </c>
-      <c r="P3" t="str">
-        <v>STATUS_TINGGAL *</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>STATUS_EKONOMI</v>
-      </c>
-      <c r="R3" t="str">
-        <v>ALAMAT_KTP</v>
-      </c>
-      <c r="S3" t="str">
-        <v>ALAMAT_DOMISILI</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>NIK *</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NO_KK *</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>NAMA_LENGKAP *</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TEMPAT_LAHIR</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>TANGGAL_LAHIR</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>JENIS_KELAMIN *</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>AGAMA</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>PENDIDIKAN</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>PEKERJAAN</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>STATUS_PERKAWINAN</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>STATUS_HUBUNGAN *</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>GOLONGAN_DARAH</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>TELEPON</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>EMAIL</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>KEWARGANEGARAAN</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>STATUS_TINGGAL *</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>STATUS_EKONOMI</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>ALAMAT_KTP</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>ALAMAT_DOMISILI</t>
+        </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>3404051705900001</v>
-      </c>
-      <c r="B4" t="str">
-        <v>3404051234567890</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Siti Aminah</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Sleman</v>
-      </c>
-      <c r="E4" t="str">
-        <v>1990-05-17</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Perempuan</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Islam</v>
-      </c>
-      <c r="H4" t="str">
-        <v>SMA</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Petani</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Kawin</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Istri</v>
-      </c>
-      <c r="L4" t="str">
-        <v>A</v>
-      </c>
-      <c r="M4" t="str">
-        <v>08129876543</v>
-      </c>
-      <c r="N4" t="str">
-        <v/>
-      </c>
-      <c r="O4" t="str">
-        <v>WNI</v>
-      </c>
-      <c r="P4" t="str">
-        <v>domisili_asli</v>
-      </c>
-      <c r="Q4" t="str">
-        <v>mampu</v>
-      </c>
-      <c r="R4" t="str">
-        <v>Jl. Majegan No.5, RT 01/01, Pandowoharjo, Sleman</v>
-      </c>
-      <c r="S4" t="str">
-        <v/>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>3404051705900001</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>3404051234567890</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Siti Aminah</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Sleman</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>1990-05-17</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Perempuan</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Islam</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>SMA</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Petani</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>Kawin</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Istri</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>08129876543</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>WNI</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>domisili_asli</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>mampu</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>Jl. Majegan No.5, RT 01/01, Pandowoharjo, Sleman</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S4"/>
-  </ignoredErrors>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>